<commit_message>
Yolias: Integrations tab back with disabled buttons and no notes; security headers; pricing study inputs (Sentry Free, domain)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/yolias-pricing-study.xlsx
+++ b/docs/yolias-pricing-study.xlsx
@@ -2085,10 +2085,10 @@
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Sentry</t>
-        </is>
-      </c>
-      <c r="B46" s="15" t="n">
+          <t>Sentry (Free)</t>
+        </is>
+      </c>
+      <c r="B46" s="13" t="n">
         <v>0</v>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -2098,7 +2098,7 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>محتاج تأكيد الخطة (محسوبة Free)</t>
+          <t>منك 2026-10-07</t>
         </is>
       </c>
     </row>
@@ -2128,8 +2128,8 @@
           <t>الدومين yolias.com — سنوياً</t>
         </is>
       </c>
-      <c r="B48" s="15" t="n">
-        <v>0</v>
+      <c r="B48" s="13" t="n">
+        <v>11.92</v>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
@@ -2138,7 +2138,7 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>محتاج سعر التجديد السنوي</t>
+          <t>منك 2026-10-07 (سعر التجديد)</t>
         </is>
       </c>
     </row>

</xml_diff>